<commit_message>
Version 3 multiples modelos
</commit_message>
<xml_diff>
--- a/Recursos/Variables_thor.xlsx
+++ b/Recursos/Variables_thor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Contratos\2025\TESIS_MINAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EEA5505-A626-417E-A5EB-CCF7DC86BF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87730006-0F16-4FE8-B7AF-A6680BAB12B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{361C9A51-F63D-4138-9444-0CEBAAD7E37D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="73">
   <si>
     <t>url</t>
   </si>
@@ -122,20 +122,146 @@
     <t>2025-03-20T21:10:52.500</t>
   </si>
   <si>
-    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHZ.D/AM.RAFDA.00.EHZ.D.2025.078</t>
-  </si>
-  <si>
-    <t>AM.RAFDA.00.EHZ.D.2025.078</t>
-  </si>
-  <si>
-    <t>2025-03-19T18:07:45.000</t>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHZ.D/AM.RAFDA.00.EHZ.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHZ.D.2025.211</t>
+  </si>
+  <si>
+    <t>2025-07-30T21:54:49.800</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHE.D/AM.R8256.00.EHE.D.2025.210</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHE.D.2025.210</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHN.D/AM.R8256.00.EHN.D.2025.210</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHN.D.2025.210</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHE.D/AM.R8256.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHN.D/AM.R8256.00.EHN.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHN.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHE.D/AM.RAFDA.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHN.D/AM.RAFDA.00.EHN.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHZ.D/AM.R0BD9.00.EHZ.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHZ.D.2025.211</t>
+  </si>
+  <si>
+    <t>2025-07-30T21:54:49.500</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/inventory/R0BD9.xml</t>
+  </si>
+  <si>
+    <t>R0BD9.xml</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHE.D/AM.R0BD9.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHE.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHN.D/AM.R0BD9.00.EHN.D.2025.211</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHN.D.2025.211</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHZ.D/AM.R0BD9.00.EHZ.D.2025.210</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHZ.D.2025.210</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHE.D/AM.R0BD9.00.EHE.D.2025.210</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHE.D.2025.210</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R0BD9/EHN.D/AM.R0BD9.00.EHN.D.2025.210</t>
+  </si>
+  <si>
+    <t>AM.R0BD9.00.EHN.D.2025.210</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHE.D/AM.RAFDA.00.EHE.D.2025.144</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHE.D.2025.144</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHN.D/AM.RAFDA.00.EHN.D.2025.144</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHN.D.2025.144</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHE.D/AM.RAFDA.00.EHE.D.2025.149</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHE.D.2025.149</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHN.D/AM.RAFDA.00.EHN.D.2025.149</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHN.D.2025.149</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHE.D/AM.RAFDA.00.EHE.D.2025.133</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHE.D.2025.133</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/RAFDA/EHN.D/AM.RAFDA.00.EHN.D.2025.133</t>
+  </si>
+  <si>
+    <t>AM.RAFDA.00.EHN.D.2025.133</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHE.D/AM.R8256.00.EHE.D.2025.079</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHE.D.2025.079</t>
+  </si>
+  <si>
+    <t>https://osso.univalle.edu.co/apps/seiscomp/archive/2025/AM/R8256/EHN.D/AM.R8256.00.EHN.D.2025.079</t>
+  </si>
+  <si>
+    <t>AM.R8256.00.EHN.D.2025.079</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,32 +270,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
+      <b/>
+      <sz val="9"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
-      <name val="open Sans"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
-      <name val="open Sans"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="open Sans"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
-      <color theme="10"/>
-      <name val="open Sans"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -189,32 +307,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -547,194 +658,628 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1B1A7EA-E10A-4FF7-98AA-FA06AF642D45}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="95.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="82.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D4" s="1">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F4" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1">
+        <v>10</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D7" s="1">
         <v>10</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="9">
-        <v>0.6</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="9">
-        <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D22" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="1">
+        <v>8</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="F23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="1">
+        <v>8</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="1">
+        <v>8</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="1">
+        <v>4</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="1">
+        <v>4</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="1">
+        <v>4</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{412F97E5-EF6C-4AC8-99FF-07619216477E}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{360634A9-DF32-4402-A02A-4D72E7E73F25}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{8275F45A-B94D-4E2C-B905-8A2681727319}"/>
-    <hyperlink ref="A4" r:id="rId4" xr:uid="{77D23CD4-935C-4095-A523-C87B96F8268B}"/>
-    <hyperlink ref="E5" r:id="rId5" xr:uid="{24C1E462-192F-49D3-B01D-D794C9F04427}"/>
-    <hyperlink ref="A5" r:id="rId6" xr:uid="{ADCA3F2B-92E2-492A-ADCC-9D7A392B1564}"/>
-    <hyperlink ref="E4" r:id="rId7" xr:uid="{E7C0DEDD-E638-4005-86DB-9D20A7C65067}"/>
-    <hyperlink ref="A6" r:id="rId8" xr:uid="{AD79E7F5-EB4A-4E67-9471-0AF21214F5B8}"/>
-    <hyperlink ref="E6" r:id="rId9" xr:uid="{A6C8BAD7-7D8D-4BD2-A803-D720A6701B77}"/>
-    <hyperlink ref="A7" r:id="rId10" xr:uid="{C1BC86D0-D7EF-4390-AD12-E0B20FE2831A}"/>
-    <hyperlink ref="E7" r:id="rId11" xr:uid="{1E287611-2F68-4322-AA31-2B2102F84A0F}"/>
-    <hyperlink ref="A8" r:id="rId12" xr:uid="{178D2E03-0A7B-4F58-9127-CAA4299A053B}"/>
-    <hyperlink ref="E8" r:id="rId13" xr:uid="{6ACF2C95-A418-4F33-AE38-B6C1D600F8DC}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId14"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>